<commit_message>
final bulkdesignation with three condition
</commit_message>
<xml_diff>
--- a/Jobs/Tasks/FileProcess/DesignationUpdateExcel.xlsx
+++ b/Jobs/Tasks/FileProcess/DesignationUpdateExcel.xlsx
@@ -38,10 +38,10 @@
     <t>AGT002</t>
   </si>
   <si>
-    <t>Branch Manager</t>
-  </si>
-  <si>
     <t>17/02/2026</t>
+  </si>
+  <si>
+    <t>Unit Manager</t>
   </si>
 </sst>
 </file>
@@ -372,7 +372,7 @@
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="9.90625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="10.6328125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="14.6328125" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="27.54296875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
@@ -392,10 +392,10 @@
         <v>3</v>
       </c>
       <c r="B2" t="s">
+        <v>5</v>
+      </c>
+      <c r="C2" t="s">
         <v>4</v>
-      </c>
-      <c r="C2" t="s">
-        <v>5</v>
       </c>
     </row>
   </sheetData>

</xml_diff>